<commit_message>
bug_fix cron quebra. Adição de flag para debug fundamentus
</commit_message>
<xml_diff>
--- a/all_ticker_financial_indicators.xlsx
+++ b/all_ticker_financial_indicators.xlsx
@@ -650,7 +650,7 @@
         </is>
       </c>
       <c r="E2" t="n">
-        <v>237260000000</v>
+        <v>242462000000</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -661,34 +661,34 @@
         <v>15763700000</v>
       </c>
       <c r="H2" t="n">
-        <v>16.16</v>
+        <v>18.54</v>
       </c>
       <c r="I2" t="n">
         <v>27.8</v>
       </c>
       <c r="J2" t="n">
-        <v>12.4</v>
+        <v>12.65</v>
       </c>
       <c r="K2" t="n">
-        <v>2.88</v>
+        <v>2.94</v>
       </c>
       <c r="L2" t="n">
-        <v>1.78</v>
+        <v>1.81</v>
       </c>
       <c r="M2" t="n">
-        <v>217.09</v>
+        <v>221.54</v>
       </c>
       <c r="N2" t="n">
-        <v>-27.88</v>
+        <v>-28.45</v>
       </c>
       <c r="O2" t="n">
-        <v>5.3</v>
+        <v>5.2</v>
       </c>
       <c r="P2" t="n">
-        <v>8.859999999999999</v>
+        <v>9.06</v>
       </c>
       <c r="Q2" t="n">
-        <v>11.59</v>
+        <v>11.84</v>
       </c>
       <c r="R2" t="n">
         <v>4.6</v>
@@ -780,7 +780,7 @@
         </is>
       </c>
       <c r="E3" t="n">
-        <v>12022200000</v>
+        <v>11850700000</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
@@ -791,34 +791,34 @@
         <v>504191000</v>
       </c>
       <c r="H3" t="n">
-        <v>3.87</v>
+        <v>2.62</v>
       </c>
       <c r="I3" t="n">
         <v>67.3</v>
       </c>
       <c r="J3" t="n">
-        <v>9.94</v>
+        <v>9.82</v>
       </c>
       <c r="K3" t="n">
-        <v>4.93</v>
+        <v>4.88</v>
       </c>
       <c r="L3" t="n">
-        <v>0.57</v>
+        <v>0.5600000000000001</v>
       </c>
       <c r="M3" t="n">
-        <v>7.5</v>
+        <v>7.41</v>
       </c>
       <c r="N3" t="n">
-        <v>-1.6</v>
+        <v>-1.58</v>
       </c>
       <c r="O3" t="n">
-        <v>9.199999999999999</v>
+        <v>9.300000000000001</v>
       </c>
       <c r="P3" t="n">
-        <v>5.84</v>
+        <v>5.75</v>
       </c>
       <c r="Q3" t="n">
-        <v>8.43</v>
+        <v>8.31</v>
       </c>
       <c r="R3" t="n">
         <v>31.3</v>
@@ -910,7 +910,7 @@
         </is>
       </c>
       <c r="E4" t="n">
-        <v>23431800000</v>
+        <v>23648400000</v>
       </c>
       <c r="F4" t="inlineStr">
         <is>
@@ -921,34 +921,34 @@
         <v>1353530000</v>
       </c>
       <c r="H4" t="n">
-        <v>17.22</v>
+        <v>19.45</v>
       </c>
       <c r="I4" t="n">
         <v>31.33</v>
       </c>
       <c r="J4" t="n">
-        <v>1.84</v>
+        <v>1.87</v>
       </c>
       <c r="K4" t="n">
         <v>0.15</v>
       </c>
       <c r="L4" t="n">
-        <v>0.24</v>
+        <v>0.25</v>
       </c>
       <c r="M4" t="n">
-        <v>7.05</v>
+        <v>7.19</v>
       </c>
       <c r="N4" t="n">
-        <v>-0.48</v>
+        <v>-0.49</v>
       </c>
       <c r="O4" t="n">
         <v>1.2</v>
       </c>
       <c r="P4" t="n">
-        <v>2.93</v>
+        <v>2.95</v>
       </c>
       <c r="Q4" t="n">
-        <v>3.77</v>
+        <v>3.81</v>
       </c>
       <c r="R4" t="n">
         <v>14.9</v>
@@ -1040,7 +1040,7 @@
         </is>
       </c>
       <c r="E5" t="n">
-        <v>33361600000</v>
+        <v>32952000000</v>
       </c>
       <c r="F5" t="inlineStr">
         <is>
@@ -1051,34 +1051,34 @@
         <v>1050380000</v>
       </c>
       <c r="H5" t="n">
-        <v>4.89</v>
+        <v>1.6</v>
       </c>
       <c r="I5" t="n">
         <v>36.25</v>
       </c>
       <c r="J5" t="n">
-        <v>11.26</v>
+        <v>10.91</v>
       </c>
       <c r="K5" t="n">
-        <v>0.98</v>
+        <v>0.95</v>
       </c>
       <c r="L5" t="n">
-        <v>0.28</v>
+        <v>0.27</v>
       </c>
       <c r="M5" t="n">
-        <v>17.72</v>
+        <v>17.16</v>
       </c>
       <c r="N5" t="n">
-        <v>-0.49</v>
+        <v>-0.47</v>
       </c>
       <c r="O5" t="n">
         <v>0</v>
       </c>
       <c r="P5" t="n">
-        <v>12.33</v>
+        <v>12.18</v>
       </c>
       <c r="Q5" t="n">
-        <v>28.74</v>
+        <v>28.38</v>
       </c>
       <c r="R5" t="n">
         <v>39.7</v>
@@ -1170,7 +1170,7 @@
         </is>
       </c>
       <c r="E6" t="n">
-        <v>203280000000</v>
+        <v>194971000000</v>
       </c>
       <c r="F6" t="inlineStr">
         <is>
@@ -1181,34 +1181,34 @@
         <v>2915430000</v>
       </c>
       <c r="H6" t="n">
-        <v>6.7</v>
+        <v>1.07</v>
       </c>
       <c r="I6" t="n">
         <v>105.25</v>
       </c>
       <c r="J6" t="n">
-        <v>21.27</v>
+        <v>20.14</v>
       </c>
       <c r="K6" t="n">
-        <v>3.61</v>
+        <v>3.42</v>
       </c>
       <c r="L6" t="n">
-        <v>0.5600000000000001</v>
+        <v>0.53</v>
       </c>
       <c r="M6" t="n">
-        <v>5.42</v>
+        <v>5.14</v>
       </c>
       <c r="N6" t="n">
-        <v>-1.52</v>
+        <v>-1.44</v>
       </c>
       <c r="O6" t="n">
-        <v>5.3</v>
+        <v>5.6</v>
       </c>
       <c r="P6" t="n">
-        <v>16.77</v>
+        <v>16.09</v>
       </c>
       <c r="Q6" t="n">
-        <v>27.46</v>
+        <v>26.34</v>
       </c>
       <c r="R6" t="n">
         <v>4.6</v>
@@ -1300,7 +1300,7 @@
         </is>
       </c>
       <c r="E7" t="n">
-        <v>218673000000</v>
+        <v>209694000000</v>
       </c>
       <c r="F7" t="inlineStr">
         <is>
@@ -1311,34 +1311,34 @@
         <v>2915430000</v>
       </c>
       <c r="H7" t="n">
-        <v>13.09</v>
+        <v>7.21</v>
       </c>
       <c r="I7" t="n">
         <v>90.78</v>
       </c>
       <c r="J7" t="n">
-        <v>23.34</v>
+        <v>22.13</v>
       </c>
       <c r="K7" t="n">
-        <v>3.97</v>
+        <v>3.76</v>
       </c>
       <c r="L7" t="n">
-        <v>0.62</v>
+        <v>0.59</v>
       </c>
       <c r="M7" t="n">
-        <v>5.95</v>
+        <v>5.64</v>
       </c>
       <c r="N7" t="n">
-        <v>-1.67</v>
+        <v>-1.58</v>
       </c>
       <c r="O7" t="n">
-        <v>5.4</v>
+        <v>5.7</v>
       </c>
       <c r="P7" t="n">
-        <v>18.04</v>
+        <v>17.3</v>
       </c>
       <c r="Q7" t="n">
-        <v>29.54</v>
+        <v>28.32</v>
       </c>
       <c r="R7" t="n">
         <v>4.6</v>
@@ -1430,7 +1430,7 @@
         </is>
       </c>
       <c r="E8" t="n">
-        <v>6459480000</v>
+        <v>6058890000</v>
       </c>
       <c r="F8" t="inlineStr">
         <is>
@@ -1441,34 +1441,34 @@
         <v>206490000</v>
       </c>
       <c r="H8" t="n">
-        <v>-17.65</v>
+        <v>-25.36</v>
       </c>
       <c r="I8" t="n">
         <v>-6.39</v>
       </c>
       <c r="J8" t="n">
-        <v>4.37</v>
+        <v>3.96</v>
       </c>
       <c r="K8" t="n">
-        <v>0.37</v>
+        <v>0.33</v>
       </c>
       <c r="L8" t="n">
-        <v>0.28</v>
+        <v>0.26</v>
       </c>
       <c r="M8" t="n">
-        <v>1.17</v>
+        <v>1.06</v>
       </c>
       <c r="N8" t="n">
-        <v>-8.630000000000001</v>
+        <v>-7.82</v>
       </c>
       <c r="O8" t="n">
-        <v>11.9</v>
+        <v>13.2</v>
       </c>
       <c r="P8" t="n">
-        <v>3.85</v>
+        <v>3.61</v>
       </c>
       <c r="Q8" t="n">
-        <v>6.6</v>
+        <v>6.19</v>
       </c>
       <c r="R8" t="n">
         <v>39.8</v>
@@ -1560,7 +1560,7 @@
         </is>
       </c>
       <c r="E9" t="n">
-        <v>83447800000</v>
+        <v>81378800000</v>
       </c>
       <c r="F9" t="inlineStr">
         <is>
@@ -1571,34 +1571,34 @@
         <v>5046500000</v>
       </c>
       <c r="H9" t="n">
-        <v>23.21</v>
+        <v>20.18</v>
       </c>
       <c r="I9" t="n">
         <v>37.23</v>
       </c>
       <c r="J9" t="n">
-        <v>11.96</v>
+        <v>11.67</v>
       </c>
       <c r="K9" t="n">
-        <v>7.21</v>
+        <v>7.03</v>
       </c>
       <c r="L9" t="n">
-        <v>1.73</v>
+        <v>1.69</v>
       </c>
       <c r="M9" t="n">
-        <v>8.970000000000001</v>
+        <v>8.75</v>
       </c>
       <c r="N9" t="n">
-        <v>-6.81</v>
+        <v>-6.64</v>
       </c>
       <c r="O9" t="n">
-        <v>3.8</v>
+        <v>3.9</v>
       </c>
       <c r="P9" t="n">
-        <v>11.26</v>
+        <v>10.98</v>
       </c>
       <c r="Q9" t="n">
-        <v>11.87</v>
+        <v>11.58</v>
       </c>
       <c r="R9" t="n">
         <v>3.2</v>
@@ -1703,7 +1703,7 @@
         <v>5730830000</v>
       </c>
       <c r="H10" t="n">
-        <v>-3.61</v>
+        <v>-7.57</v>
       </c>
       <c r="I10" t="n">
         <v>-5.56</v>
@@ -1734,7 +1734,7 @@
         </is>
       </c>
       <c r="O10" t="n">
-        <v>4</v>
+        <v>4.1</v>
       </c>
       <c r="P10" t="inlineStr">
         <is>
@@ -1857,7 +1857,7 @@
         <v>10592000000</v>
       </c>
       <c r="H11" t="n">
-        <v>0.57</v>
+        <v>-0.27</v>
       </c>
       <c r="I11" t="n">
         <v>62.17</v>
@@ -1888,7 +1888,7 @@
         </is>
       </c>
       <c r="O11" t="n">
-        <v>8.9</v>
+        <v>9</v>
       </c>
       <c r="P11" t="inlineStr">
         <is>
@@ -2011,7 +2011,7 @@
         <v>10592000000</v>
       </c>
       <c r="H12" t="n">
-        <v>-1.51</v>
+        <v>-2.18</v>
       </c>
       <c r="I12" t="n">
         <v>73.45999999999999</v>
@@ -2042,7 +2042,7 @@
         </is>
       </c>
       <c r="O12" t="n">
-        <v>8.5</v>
+        <v>8.6</v>
       </c>
       <c r="P12" t="inlineStr">
         <is>
@@ -2165,13 +2165,13 @@
         <v>1941400000</v>
       </c>
       <c r="H13" t="n">
-        <v>2.36</v>
+        <v>4.03</v>
       </c>
       <c r="I13" t="n">
         <v>12.22</v>
       </c>
       <c r="J13" t="n">
-        <v>6.69</v>
+        <v>6.8</v>
       </c>
       <c r="K13" t="inlineStr">
         <is>
@@ -2179,7 +2179,7 @@
         </is>
       </c>
       <c r="L13" t="n">
-        <v>3.41</v>
+        <v>3.47</v>
       </c>
       <c r="M13" t="inlineStr">
         <is>
@@ -2192,7 +2192,7 @@
         </is>
       </c>
       <c r="O13" t="n">
-        <v>13.6</v>
+        <v>13.3</v>
       </c>
       <c r="P13" t="inlineStr">
         <is>
@@ -2308,7 +2308,7 @@
         </is>
       </c>
       <c r="E14" t="n">
-        <v>17472400000</v>
+        <v>17192200000</v>
       </c>
       <c r="F14" t="inlineStr">
         <is>
@@ -2319,34 +2319,34 @@
         <v>1000540000</v>
       </c>
       <c r="H14" t="n">
-        <v>-33.85</v>
+        <v>-38.75</v>
       </c>
       <c r="I14" t="n">
         <v>43.81</v>
       </c>
       <c r="J14" t="n">
-        <v>0.97</v>
+        <v>0.9</v>
       </c>
       <c r="K14" t="n">
-        <v>0.07000000000000001</v>
+        <v>0.06</v>
       </c>
       <c r="L14" t="n">
-        <v>0.09</v>
+        <v>0.08</v>
       </c>
       <c r="M14" t="n">
-        <v>0.65</v>
+        <v>0.6</v>
       </c>
       <c r="N14" t="n">
-        <v>-0.24</v>
+        <v>-0.23</v>
       </c>
       <c r="O14" t="n">
-        <v>5.2</v>
+        <v>5.6</v>
       </c>
       <c r="P14" t="n">
-        <v>3.56</v>
+        <v>3.51</v>
       </c>
       <c r="Q14" t="n">
-        <v>4.47</v>
+        <v>4.4</v>
       </c>
       <c r="R14" t="n">
         <v>17.7</v>
@@ -2451,7 +2451,7 @@
         <v>11670100000</v>
       </c>
       <c r="H15" t="n">
-        <v>2.57</v>
+        <v>0.32</v>
       </c>
       <c r="I15" t="n">
         <v>98.73999999999999</v>
@@ -2592,7 +2592,7 @@
         </is>
       </c>
       <c r="E16" t="n">
-        <v>8852060000</v>
+        <v>8734130000</v>
       </c>
       <c r="F16" t="inlineStr">
         <is>
@@ -2603,13 +2603,13 @@
         <v>393097000</v>
       </c>
       <c r="H16" t="n">
-        <v>16.43</v>
+        <v>14.92</v>
       </c>
       <c r="I16" t="n">
         <v>40.74</v>
       </c>
       <c r="J16" t="n">
-        <v>-253.86</v>
+        <v>-250.57</v>
       </c>
       <c r="K16" t="inlineStr">
         <is>
@@ -2617,22 +2617,22 @@
         </is>
       </c>
       <c r="L16" t="n">
-        <v>1.16</v>
+        <v>1.14</v>
       </c>
       <c r="M16" t="n">
-        <v>42.63</v>
+        <v>42.07</v>
       </c>
       <c r="N16" t="n">
-        <v>43.38</v>
+        <v>42.81</v>
       </c>
       <c r="O16" t="n">
-        <v>10.2</v>
+        <v>10.3</v>
       </c>
       <c r="P16" t="n">
-        <v>-246.72</v>
+        <v>-243.43</v>
       </c>
       <c r="Q16" t="n">
-        <v>-246.72</v>
+        <v>-243.43</v>
       </c>
       <c r="R16" t="inlineStr">
         <is>
@@ -2732,7 +2732,7 @@
         </is>
       </c>
       <c r="E17" t="n">
-        <v>19816300000</v>
+        <v>20276300000</v>
       </c>
       <c r="F17" t="inlineStr">
         <is>
@@ -2743,34 +2743,34 @@
         <v>464557000</v>
       </c>
       <c r="H17" t="n">
-        <v>18.16</v>
+        <v>24.08</v>
       </c>
       <c r="I17" t="n">
         <v>-28.4</v>
       </c>
       <c r="J17" t="n">
-        <v>3.27</v>
+        <v>3.44</v>
       </c>
       <c r="K17" t="n">
-        <v>0.77</v>
+        <v>0.8100000000000001</v>
       </c>
       <c r="L17" t="n">
-        <v>0.22</v>
+        <v>0.23</v>
       </c>
       <c r="M17" t="n">
-        <v>10.25</v>
+        <v>10.76</v>
       </c>
       <c r="N17" t="n">
-        <v>-0.4</v>
+        <v>-0.42</v>
       </c>
       <c r="O17" t="n">
         <v>0.6</v>
       </c>
       <c r="P17" t="n">
-        <v>3.58</v>
+        <v>3.67</v>
       </c>
       <c r="Q17" t="n">
-        <v>7.06</v>
+        <v>7.22</v>
       </c>
       <c r="R17" t="n">
         <v>93.8</v>
@@ -2862,7 +2862,7 @@
         </is>
       </c>
       <c r="E18" t="n">
-        <v>52560600000</v>
+        <v>51173400000</v>
       </c>
       <c r="F18" t="inlineStr">
         <is>
@@ -2873,34 +2873,34 @@
         <v>797208000</v>
       </c>
       <c r="H18" t="n">
-        <v>51.71</v>
+        <v>29.66</v>
       </c>
       <c r="I18" t="n">
         <v>-31.87</v>
       </c>
       <c r="J18" t="n">
-        <v>-2.51</v>
+        <v>-2.14</v>
       </c>
       <c r="K18" t="n">
-        <v>0.14</v>
+        <v>0.12</v>
       </c>
       <c r="L18" t="n">
-        <v>0.13</v>
+        <v>0.11</v>
       </c>
       <c r="M18" t="n">
-        <v>-0.89</v>
+        <v>-0.76</v>
       </c>
       <c r="N18" t="n">
-        <v>-0.14</v>
+        <v>-0.12</v>
       </c>
       <c r="O18" t="n">
         <v>0</v>
       </c>
       <c r="P18" t="n">
-        <v>61.76</v>
+        <v>60.13</v>
       </c>
       <c r="Q18" t="n">
-        <v>-13.82</v>
+        <v>-13.45</v>
       </c>
       <c r="R18" t="n">
         <v>-10.6</v>
@@ -2992,7 +2992,7 @@
         </is>
       </c>
       <c r="E19" t="n">
-        <v>3580920000</v>
+        <v>3624070000</v>
       </c>
       <c r="F19" t="inlineStr">
         <is>
@@ -3003,34 +3003,34 @@
         <v>308245000</v>
       </c>
       <c r="H19" t="n">
-        <v>-12.3</v>
+        <v>-11.21</v>
       </c>
       <c r="I19" t="n">
         <v>70.75</v>
       </c>
       <c r="J19" t="n">
-        <v>3.61</v>
+        <v>3.66</v>
       </c>
       <c r="K19" t="n">
-        <v>0.43</v>
+        <v>0.44</v>
       </c>
       <c r="L19" t="n">
         <v>0.4</v>
       </c>
       <c r="M19" t="n">
-        <v>2.14</v>
+        <v>2.17</v>
       </c>
       <c r="N19" t="n">
-        <v>-3.78</v>
+        <v>-3.83</v>
       </c>
       <c r="O19" t="n">
-        <v>4.7</v>
+        <v>4.6</v>
       </c>
       <c r="P19" t="n">
-        <v>2.75</v>
+        <v>2.78</v>
       </c>
       <c r="Q19" t="n">
-        <v>3.75</v>
+        <v>3.8</v>
       </c>
       <c r="R19" t="n">
         <v>9.9</v>
@@ -3122,7 +3122,7 @@
         </is>
       </c>
       <c r="E20" t="n">
-        <v>49927200000</v>
+        <v>48753900000</v>
       </c>
       <c r="F20" t="inlineStr">
         <is>
@@ -3133,34 +3133,34 @@
         <v>2861780000</v>
       </c>
       <c r="H20" t="n">
-        <v>3.69</v>
+        <v>-0.1</v>
       </c>
       <c r="I20" t="n">
         <v>16.12</v>
       </c>
       <c r="J20" t="n">
-        <v>5.28</v>
+        <v>5.09</v>
       </c>
       <c r="K20" t="n">
-        <v>0.74</v>
+        <v>0.71</v>
       </c>
       <c r="L20" t="n">
-        <v>0.47</v>
+        <v>0.45</v>
       </c>
       <c r="M20" t="n">
-        <v>-30.26</v>
+        <v>-29.15</v>
       </c>
       <c r="N20" t="n">
-        <v>-1.29</v>
+        <v>-1.24</v>
       </c>
       <c r="O20" t="n">
-        <v>8.4</v>
+        <v>8.699999999999999</v>
       </c>
       <c r="P20" t="n">
-        <v>6.53</v>
+        <v>6.37</v>
       </c>
       <c r="Q20" t="n">
-        <v>8.210000000000001</v>
+        <v>8.02</v>
       </c>
       <c r="R20" t="n">
         <v>6.2</v>
@@ -3252,7 +3252,7 @@
         </is>
       </c>
       <c r="E21" t="n">
-        <v>24604200000</v>
+        <v>24930100000</v>
       </c>
       <c r="F21" t="inlineStr">
         <is>
@@ -3263,34 +3263,34 @@
         <v>5432040000</v>
       </c>
       <c r="H21" t="n">
-        <v>-14.21</v>
+        <v>-13.06</v>
       </c>
       <c r="I21" t="n">
         <v>13.91</v>
       </c>
       <c r="J21" t="n">
-        <v>4.75</v>
+        <v>4.81</v>
       </c>
       <c r="K21" t="n">
-        <v>1.37</v>
+        <v>1.38</v>
       </c>
       <c r="L21" t="n">
-        <v>0.71</v>
+        <v>0.72</v>
       </c>
       <c r="M21" t="n">
-        <v>7.05</v>
+        <v>7.14</v>
       </c>
       <c r="N21" t="n">
-        <v>-1.69</v>
+        <v>-1.71</v>
       </c>
       <c r="O21" t="n">
-        <v>24.3</v>
+        <v>24</v>
       </c>
       <c r="P21" t="n">
-        <v>3.82</v>
+        <v>3.87</v>
       </c>
       <c r="Q21" t="n">
-        <v>4.8</v>
+        <v>4.86</v>
       </c>
       <c r="R21" t="n">
         <v>2.6</v>
@@ -3382,7 +3382,7 @@
         </is>
       </c>
       <c r="E22" t="n">
-        <v>10388500000</v>
+        <v>10429800000</v>
       </c>
       <c r="F22" t="inlineStr">
         <is>
@@ -3393,22 +3393,22 @@
         <v>2064270000</v>
       </c>
       <c r="H22" t="n">
-        <v>-22.09</v>
+        <v>-21.45</v>
       </c>
       <c r="I22" t="n">
         <v>238.23</v>
       </c>
       <c r="J22" t="n">
-        <v>2.31</v>
+        <v>2.33</v>
       </c>
       <c r="K22" t="n">
-        <v>0.67</v>
+        <v>0.68</v>
       </c>
       <c r="L22" t="n">
         <v>0.21</v>
       </c>
       <c r="M22" t="n">
-        <v>2.57</v>
+        <v>2.59</v>
       </c>
       <c r="N22" t="n">
         <v>-0.89</v>
@@ -3417,10 +3417,10 @@
         <v>4.8</v>
       </c>
       <c r="P22" t="n">
-        <v>3.61</v>
+        <v>3.63</v>
       </c>
       <c r="Q22" t="n">
-        <v>4.74</v>
+        <v>4.76</v>
       </c>
       <c r="R22" t="n">
         <v>11.6</v>
@@ -3512,7 +3512,7 @@
         </is>
       </c>
       <c r="E23" t="n">
-        <v>75866400000</v>
+        <v>75336300000</v>
       </c>
       <c r="F23" t="inlineStr">
         <is>
@@ -3523,34 +3523,34 @@
         <v>1152250000</v>
       </c>
       <c r="H23" t="n">
-        <v>-12.26</v>
+        <v>-13.2</v>
       </c>
       <c r="I23" t="n">
         <v>81.66</v>
       </c>
       <c r="J23" t="n">
-        <v>4.38</v>
+        <v>4.34</v>
       </c>
       <c r="K23" t="n">
-        <v>1.11</v>
+        <v>1.1</v>
       </c>
       <c r="L23" t="n">
         <v>0.59</v>
       </c>
       <c r="M23" t="n">
-        <v>19.92</v>
+        <v>19.71</v>
       </c>
       <c r="N23" t="n">
-        <v>-1.28</v>
+        <v>-1.27</v>
       </c>
       <c r="O23" t="n">
-        <v>8.6</v>
+        <v>8.699999999999999</v>
       </c>
       <c r="P23" t="n">
-        <v>5.63</v>
+        <v>5.59</v>
       </c>
       <c r="Q23" t="n">
-        <v>6.66</v>
+        <v>6.62</v>
       </c>
       <c r="R23" t="n">
         <v>3.1</v>
@@ -3642,7 +3642,7 @@
         </is>
       </c>
       <c r="E24" t="n">
-        <v>62076100000</v>
+        <v>61121600000</v>
       </c>
       <c r="F24" t="inlineStr">
         <is>
@@ -3653,34 +3653,34 @@
         <v>2982810000</v>
       </c>
       <c r="H24" t="n">
-        <v>21.16</v>
+        <v>18.53</v>
       </c>
       <c r="I24" t="n">
         <v>64.94</v>
       </c>
       <c r="J24" t="n">
-        <v>9</v>
+        <v>8.800000000000001</v>
       </c>
       <c r="K24" t="n">
-        <v>1.61</v>
+        <v>1.57</v>
       </c>
       <c r="L24" t="n">
-        <v>0.7</v>
+        <v>0.68</v>
       </c>
       <c r="M24" t="n">
-        <v>12.38</v>
+        <v>12.11</v>
       </c>
       <c r="N24" t="n">
-        <v>-1.69</v>
+        <v>-1.65</v>
       </c>
       <c r="O24" t="n">
-        <v>7.2</v>
+        <v>7.4</v>
       </c>
       <c r="P24" t="n">
-        <v>9.68</v>
+        <v>9.529999999999999</v>
       </c>
       <c r="Q24" t="n">
-        <v>12.71</v>
+        <v>12.52</v>
       </c>
       <c r="R24" t="n">
         <v>2.7</v>
@@ -3772,7 +3772,7 @@
         </is>
       </c>
       <c r="E25" t="n">
-        <v>64429200000</v>
+        <v>62802900000</v>
       </c>
       <c r="F25" t="inlineStr">
         <is>
@@ -3783,34 +3783,34 @@
         <v>3966570000</v>
       </c>
       <c r="H25" t="n">
-        <v>-19.36</v>
+        <v>-27.07</v>
       </c>
       <c r="I25" t="n">
         <v>-34.8</v>
       </c>
       <c r="J25" t="n">
-        <v>1.89</v>
+        <v>1.71</v>
       </c>
       <c r="K25" t="n">
-        <v>0.43</v>
+        <v>0.39</v>
       </c>
       <c r="L25" t="n">
-        <v>0.13</v>
+        <v>0.12</v>
       </c>
       <c r="M25" t="n">
-        <v>1.15</v>
+        <v>1.04</v>
       </c>
       <c r="N25" t="n">
-        <v>-0.26</v>
+        <v>-0.23</v>
       </c>
       <c r="O25" t="n">
         <v>0</v>
       </c>
       <c r="P25" t="n">
-        <v>5</v>
+        <v>4.88</v>
       </c>
       <c r="Q25" t="n">
-        <v>7.17</v>
+        <v>6.99</v>
       </c>
       <c r="R25" t="n">
         <v>7.8</v>
@@ -3902,7 +3902,7 @@
         </is>
       </c>
       <c r="E26" t="n">
-        <v>26745900000</v>
+        <v>26711600000</v>
       </c>
       <c r="F26" t="inlineStr">
         <is>
@@ -3913,22 +3913,22 @@
         <v>380253000</v>
       </c>
       <c r="H26" t="n">
-        <v>19.89</v>
+        <v>19.69</v>
       </c>
       <c r="I26" t="n">
         <v>124.98</v>
       </c>
       <c r="J26" t="n">
-        <v>9.220000000000001</v>
+        <v>9.210000000000001</v>
       </c>
       <c r="K26" t="n">
-        <v>2.37</v>
+        <v>2.36</v>
       </c>
       <c r="L26" t="n">
-        <v>0.93</v>
+        <v>0.92</v>
       </c>
       <c r="M26" t="n">
-        <v>12.38</v>
+        <v>12.36</v>
       </c>
       <c r="N26" t="n">
         <v>-2.35</v>
@@ -3937,10 +3937,10 @@
         <v>4.3</v>
       </c>
       <c r="P26" t="n">
-        <v>8.52</v>
+        <v>8.51</v>
       </c>
       <c r="Q26" t="n">
-        <v>12.4</v>
+        <v>12.39</v>
       </c>
       <c r="R26" t="n">
         <v>9.5</v>
@@ -4032,7 +4032,7 @@
         </is>
       </c>
       <c r="E27" t="n">
-        <v>45920200000</v>
+        <v>45681500000</v>
       </c>
       <c r="F27" t="inlineStr">
         <is>
@@ -4043,13 +4043,13 @@
         <v>1326090000</v>
       </c>
       <c r="H27" t="n">
-        <v>-24.72</v>
+        <v>-26.73</v>
       </c>
       <c r="I27" t="n">
         <v>0.9</v>
       </c>
       <c r="J27" t="n">
-        <v>1.41</v>
+        <v>1.38</v>
       </c>
       <c r="K27" t="n">
         <v>0.2</v>
@@ -4058,19 +4058,19 @@
         <v>0.09</v>
       </c>
       <c r="M27" t="n">
-        <v>3.07</v>
+        <v>2.98</v>
       </c>
       <c r="N27" t="n">
-        <v>-0.17</v>
+        <v>-0.16</v>
       </c>
       <c r="O27" t="n">
         <v>0</v>
       </c>
       <c r="P27" t="n">
-        <v>4.32</v>
+        <v>4.3</v>
       </c>
       <c r="Q27" t="n">
-        <v>7.28</v>
+        <v>7.24</v>
       </c>
       <c r="R27" t="n">
         <v>-1.2</v>
@@ -4162,7 +4162,7 @@
         </is>
       </c>
       <c r="E28" t="n">
-        <v>8997800000</v>
+        <v>9241160000</v>
       </c>
       <c r="F28" t="inlineStr">
         <is>
@@ -4173,34 +4173,34 @@
         <v>308048000</v>
       </c>
       <c r="H28" t="n">
-        <v>-2.39</v>
+        <v>0.14</v>
       </c>
       <c r="I28" t="n">
         <v>113.17</v>
       </c>
       <c r="J28" t="n">
-        <v>6.11</v>
+        <v>6.27</v>
       </c>
       <c r="K28" t="n">
-        <v>1.62</v>
+        <v>1.66</v>
       </c>
       <c r="L28" t="n">
-        <v>1.52</v>
+        <v>1.56</v>
       </c>
       <c r="M28" t="n">
-        <v>5.26</v>
+        <v>5.39</v>
       </c>
       <c r="N28" t="n">
-        <v>-15.38</v>
+        <v>-15.77</v>
       </c>
       <c r="O28" t="n">
-        <v>13.7</v>
+        <v>13.4</v>
       </c>
       <c r="P28" t="n">
-        <v>5.72</v>
+        <v>5.87</v>
       </c>
       <c r="Q28" t="n">
-        <v>5.84</v>
+        <v>6</v>
       </c>
       <c r="R28" t="n">
         <v>33.2</v>
@@ -4292,7 +4292,7 @@
         </is>
       </c>
       <c r="E29" t="n">
-        <v>51340600000</v>
+        <v>51250600000</v>
       </c>
       <c r="F29" t="inlineStr">
         <is>
@@ -4303,13 +4303,13 @@
         <v>3000000000</v>
       </c>
       <c r="H29" t="n">
-        <v>9.449999999999999</v>
+        <v>9.27</v>
       </c>
       <c r="I29" t="n">
         <v>27.12</v>
       </c>
       <c r="J29" t="n">
-        <v>-332.15</v>
+        <v>-331.58</v>
       </c>
       <c r="K29" t="inlineStr">
         <is>
@@ -4320,19 +4320,19 @@
         <v>3.51</v>
       </c>
       <c r="M29" t="n">
-        <v>53.58</v>
+        <v>53.49</v>
       </c>
       <c r="N29" t="n">
-        <v>54.25</v>
+        <v>54.16</v>
       </c>
       <c r="O29" t="n">
         <v>7.5</v>
       </c>
       <c r="P29" t="n">
-        <v>-328.67</v>
+        <v>-328.1</v>
       </c>
       <c r="Q29" t="n">
-        <v>-325.19</v>
+        <v>-324.62</v>
       </c>
       <c r="R29" t="inlineStr">
         <is>
@@ -4432,7 +4432,7 @@
         </is>
       </c>
       <c r="E30" t="n">
-        <v>14631100000</v>
+        <v>15147300000</v>
       </c>
       <c r="F30" t="inlineStr">
         <is>
@@ -4443,34 +4443,34 @@
         <v>456800000</v>
       </c>
       <c r="H30" t="n">
-        <v>-14.65</v>
+        <v>-10.12</v>
       </c>
       <c r="I30" t="n">
         <v>97.78</v>
       </c>
       <c r="J30" t="n">
-        <v>6.24</v>
+        <v>6.57</v>
       </c>
       <c r="K30" t="n">
-        <v>1.02</v>
+        <v>1.08</v>
       </c>
       <c r="L30" t="n">
-        <v>0.36</v>
+        <v>0.38</v>
       </c>
       <c r="M30" t="n">
-        <v>0.87</v>
+        <v>0.92</v>
       </c>
       <c r="N30" t="n">
-        <v>27.15</v>
+        <v>28.59</v>
       </c>
       <c r="O30" t="n">
-        <v>10.8</v>
+        <v>10.3</v>
       </c>
       <c r="P30" t="n">
-        <v>8.56</v>
+        <v>8.859999999999999</v>
       </c>
       <c r="Q30" t="n">
-        <v>9.41</v>
+        <v>9.74</v>
       </c>
       <c r="R30" t="n">
         <v>18.5</v>
@@ -4562,7 +4562,7 @@
         </is>
       </c>
       <c r="E31" t="n">
-        <v>7415400000</v>
+        <v>7701680000</v>
       </c>
       <c r="F31" t="inlineStr">
         <is>
@@ -4573,34 +4573,34 @@
         <v>520500000</v>
       </c>
       <c r="H31" t="n">
-        <v>-9.210000000000001</v>
+        <v>-5.31</v>
       </c>
       <c r="I31" t="n">
         <v>93.63</v>
       </c>
       <c r="J31" t="n">
-        <v>5.84</v>
+        <v>6.09</v>
       </c>
       <c r="K31" t="n">
-        <v>1.45</v>
+        <v>1.51</v>
       </c>
       <c r="L31" t="n">
-        <v>0.48</v>
+        <v>0.5</v>
       </c>
       <c r="M31" t="n">
-        <v>1.31</v>
+        <v>1.36</v>
       </c>
       <c r="N31" t="n">
-        <v>-1.42</v>
+        <v>-1.48</v>
       </c>
       <c r="O31" t="n">
-        <v>17.3</v>
+        <v>16.6</v>
       </c>
       <c r="P31" t="n">
-        <v>6.04</v>
+        <v>6.27</v>
       </c>
       <c r="Q31" t="n">
-        <v>6.49</v>
+        <v>6.74</v>
       </c>
       <c r="R31" t="n">
         <v>26</v>
@@ -4692,7 +4692,7 @@
         </is>
       </c>
       <c r="E32" t="n">
-        <v>61623900000</v>
+        <v>62183700000</v>
       </c>
       <c r="F32" t="inlineStr">
         <is>
@@ -4703,34 +4703,34 @@
         <v>1142300000</v>
       </c>
       <c r="H32" t="n">
-        <v>4.45</v>
+        <v>6.04</v>
       </c>
       <c r="I32" t="n">
         <v>29.55</v>
       </c>
       <c r="J32" t="n">
-        <v>6.5</v>
+        <v>6.6</v>
       </c>
       <c r="K32" t="n">
-        <v>2.78</v>
+        <v>2.83</v>
       </c>
       <c r="L32" t="n">
-        <v>0.63</v>
+        <v>0.64</v>
       </c>
       <c r="M32" t="n">
-        <v>10.59</v>
+        <v>10.75</v>
       </c>
       <c r="N32" t="n">
-        <v>-1.09</v>
+        <v>-1.1</v>
       </c>
       <c r="O32" t="n">
         <v>3.7</v>
       </c>
       <c r="P32" t="n">
-        <v>8.640000000000001</v>
+        <v>8.720000000000001</v>
       </c>
       <c r="Q32" t="n">
-        <v>10.86</v>
+        <v>10.96</v>
       </c>
       <c r="R32" t="n">
         <v>1.3</v>
@@ -4822,7 +4822,7 @@
         </is>
       </c>
       <c r="E33" t="n">
-        <v>56560900000</v>
+        <v>56442400000</v>
       </c>
       <c r="F33" t="inlineStr">
         <is>
@@ -4833,13 +4833,13 @@
         <v>740465000</v>
       </c>
       <c r="H33" t="n">
-        <v>-18.36</v>
+        <v>-18.54</v>
       </c>
       <c r="I33" t="n">
         <v>58.97</v>
       </c>
       <c r="J33" t="n">
-        <v>11.8</v>
+        <v>11.77</v>
       </c>
       <c r="K33" t="n">
         <v>1.24</v>
@@ -4848,19 +4848,19 @@
         <v>0.79</v>
       </c>
       <c r="M33" t="n">
-        <v>4.4</v>
+        <v>4.39</v>
       </c>
       <c r="N33" t="n">
-        <v>-4.86</v>
+        <v>-4.85</v>
       </c>
       <c r="O33" t="n">
         <v>1</v>
       </c>
       <c r="P33" t="n">
-        <v>9.48</v>
+        <v>9.460000000000001</v>
       </c>
       <c r="Q33" t="n">
-        <v>12.46</v>
+        <v>12.43</v>
       </c>
       <c r="R33" t="n">
         <v>20.3</v>
@@ -4952,7 +4952,7 @@
         </is>
       </c>
       <c r="E34" t="n">
-        <v>66815000000</v>
+        <v>66660000000</v>
       </c>
       <c r="F34" t="inlineStr">
         <is>
@@ -4963,34 +4963,34 @@
         <v>1937030000</v>
       </c>
       <c r="H34" t="n">
-        <v>23.69</v>
+        <v>23.29</v>
       </c>
       <c r="I34" t="n">
         <v>91.64</v>
       </c>
       <c r="J34" t="n">
-        <v>14.88</v>
+        <v>14.83</v>
       </c>
       <c r="K34" t="n">
-        <v>2.59</v>
+        <v>2.58</v>
       </c>
       <c r="L34" t="n">
         <v>0.82</v>
       </c>
       <c r="M34" t="n">
-        <v>14.57</v>
+        <v>14.52</v>
       </c>
       <c r="N34" t="n">
-        <v>-1.84</v>
+        <v>-1.83</v>
       </c>
       <c r="O34" t="n">
         <v>0</v>
       </c>
       <c r="P34" t="n">
-        <v>11.04</v>
+        <v>11.02</v>
       </c>
       <c r="Q34" t="n">
-        <v>20.56</v>
+        <v>20.52</v>
       </c>
       <c r="R34" t="n">
         <v>38.1</v>
@@ -5082,7 +5082,7 @@
         </is>
       </c>
       <c r="E35" t="n">
-        <v>57923200000</v>
+        <v>57928200000</v>
       </c>
       <c r="F35" t="inlineStr">
         <is>
@@ -5093,7 +5093,7 @@
         <v>2518370000</v>
       </c>
       <c r="H35" t="n">
-        <v>1.59</v>
+        <v>1.61</v>
       </c>
       <c r="I35" t="n">
         <v>54.07</v>
@@ -5212,7 +5212,7 @@
         </is>
       </c>
       <c r="E36" t="n">
-        <v>93383300000</v>
+        <v>94340300000</v>
       </c>
       <c r="F36" t="inlineStr">
         <is>
@@ -5223,34 +5223,34 @@
         <v>1259240000</v>
       </c>
       <c r="H36" t="n">
-        <v>-2.16</v>
+        <v>-0.18</v>
       </c>
       <c r="I36" t="n">
         <v>48.71</v>
       </c>
       <c r="J36" t="n">
-        <v>4.84</v>
+        <v>4.94</v>
       </c>
       <c r="K36" t="n">
-        <v>0.89</v>
+        <v>0.91</v>
       </c>
       <c r="L36" t="n">
-        <v>0.42</v>
+        <v>0.43</v>
       </c>
       <c r="M36" t="n">
-        <v>4.85</v>
+        <v>4.95</v>
       </c>
       <c r="N36" t="n">
-        <v>-0.84</v>
+        <v>-0.86</v>
       </c>
       <c r="O36" t="n">
-        <v>4.2</v>
+        <v>4.1</v>
       </c>
       <c r="P36" t="n">
-        <v>7.31</v>
+        <v>7.38</v>
       </c>
       <c r="Q36" t="n">
-        <v>9.529999999999999</v>
+        <v>9.619999999999999</v>
       </c>
       <c r="R36" t="n">
         <v>20.2</v>
@@ -5342,7 +5342,7 @@
         </is>
       </c>
       <c r="E37" t="n">
-        <v>11792300000</v>
+        <v>11584300000</v>
       </c>
       <c r="F37" t="inlineStr">
         <is>
@@ -5353,34 +5353,34 @@
         <v>547191000</v>
       </c>
       <c r="H37" t="n">
-        <v>4.6</v>
+        <v>2.07</v>
       </c>
       <c r="I37" t="n">
         <v>39.4</v>
       </c>
       <c r="J37" t="n">
-        <v>6.68</v>
+        <v>6.52</v>
       </c>
       <c r="K37" t="n">
-        <v>1.01</v>
+        <v>0.99</v>
       </c>
       <c r="L37" t="n">
-        <v>0.64</v>
+        <v>0.63</v>
       </c>
       <c r="M37" t="n">
-        <v>3.47</v>
+        <v>3.39</v>
       </c>
       <c r="N37" t="n">
-        <v>-2.53</v>
+        <v>-2.47</v>
       </c>
       <c r="O37" t="n">
-        <v>6.9</v>
+        <v>7</v>
       </c>
       <c r="P37" t="n">
-        <v>5.34</v>
+        <v>5.25</v>
       </c>
       <c r="Q37" t="n">
-        <v>9.17</v>
+        <v>9.01</v>
       </c>
       <c r="R37" t="n">
         <v>22.1</v>
@@ -5472,7 +5472,7 @@
         </is>
       </c>
       <c r="E38" t="n">
-        <v>55908200000</v>
+        <v>54181100000</v>
       </c>
       <c r="F38" t="inlineStr">
         <is>
@@ -5483,34 +5483,34 @@
         <v>1985160000</v>
       </c>
       <c r="H38" t="n">
-        <v>19.29</v>
+        <v>14.97</v>
       </c>
       <c r="I38" t="n">
         <v>16.53</v>
       </c>
       <c r="J38" t="n">
-        <v>7.67</v>
+        <v>7.39</v>
       </c>
       <c r="K38" t="n">
-        <v>0.6899999999999999</v>
+        <v>0.66</v>
       </c>
       <c r="L38" t="n">
-        <v>0.59</v>
+        <v>0.57</v>
       </c>
       <c r="M38" t="n">
-        <v>2.62</v>
+        <v>2.52</v>
       </c>
       <c r="N38" t="n">
-        <v>95.70999999999999</v>
+        <v>92.25</v>
       </c>
       <c r="O38" t="n">
-        <v>2.9</v>
+        <v>3</v>
       </c>
       <c r="P38" t="n">
-        <v>5.63</v>
+        <v>5.46</v>
       </c>
       <c r="Q38" t="n">
-        <v>9</v>
+        <v>8.720000000000001</v>
       </c>
       <c r="R38" t="n">
         <v>-5.1</v>
@@ -5602,7 +5602,7 @@
         </is>
       </c>
       <c r="E39" t="n">
-        <v>22023100000</v>
+        <v>21453400000</v>
       </c>
       <c r="F39" t="inlineStr">
         <is>
@@ -5613,34 +5613,34 @@
         <v>1324910000</v>
       </c>
       <c r="H39" t="n">
-        <v>17.38</v>
+        <v>12.53</v>
       </c>
       <c r="I39" t="n">
         <v>21.97</v>
       </c>
       <c r="J39" t="n">
-        <v>2.23</v>
+        <v>2.13</v>
       </c>
       <c r="K39" t="n">
-        <v>0.2</v>
+        <v>0.19</v>
       </c>
       <c r="L39" t="n">
-        <v>0.17</v>
+        <v>0.16</v>
       </c>
       <c r="M39" t="n">
-        <v>0.76</v>
+        <v>0.72</v>
       </c>
       <c r="N39" t="n">
-        <v>24.64</v>
+        <v>23.63</v>
       </c>
       <c r="O39" t="n">
-        <v>3.2</v>
+        <v>3.3</v>
       </c>
       <c r="P39" t="n">
-        <v>2.22</v>
+        <v>2.16</v>
       </c>
       <c r="Q39" t="n">
-        <v>3.55</v>
+        <v>3.46</v>
       </c>
       <c r="R39" t="n">
         <v>-5.1</v>
@@ -5732,7 +5732,7 @@
         </is>
       </c>
       <c r="E40" t="n">
-        <v>11030200000</v>
+        <v>11105600000</v>
       </c>
       <c r="F40" t="inlineStr">
         <is>
@@ -5743,13 +5743,13 @@
         <v>502631000</v>
       </c>
       <c r="H40" t="n">
-        <v>-18.19</v>
+        <v>-17.18</v>
       </c>
       <c r="I40" t="n">
         <v>-55.96</v>
       </c>
       <c r="J40" t="n">
-        <v>5.51</v>
+        <v>5.58</v>
       </c>
       <c r="K40" t="n">
         <v>0.19</v>
@@ -5758,19 +5758,19 @@
         <v>0.08</v>
       </c>
       <c r="M40" t="n">
-        <v>1.22</v>
+        <v>1.24</v>
       </c>
       <c r="N40" t="n">
-        <v>-0.44</v>
+        <v>-0.45</v>
       </c>
       <c r="O40" t="n">
         <v>0</v>
       </c>
       <c r="P40" t="n">
-        <v>5.97</v>
+        <v>6.01</v>
       </c>
       <c r="Q40" t="n">
-        <v>10.04</v>
+        <v>10.11</v>
       </c>
       <c r="R40" t="n">
         <v>25.1</v>
@@ -5862,7 +5862,7 @@
         </is>
       </c>
       <c r="E41" t="n">
-        <v>22115200000</v>
+        <v>21319700000</v>
       </c>
       <c r="F41" t="inlineStr">
         <is>
@@ -5873,34 +5873,34 @@
         <v>704009000</v>
       </c>
       <c r="H41" t="n">
-        <v>-2.36</v>
+        <v>-7.25</v>
       </c>
       <c r="I41" t="n">
         <v>36</v>
       </c>
       <c r="J41" t="n">
-        <v>6.45</v>
+        <v>6.13</v>
       </c>
       <c r="K41" t="n">
-        <v>1.84</v>
+        <v>1.75</v>
       </c>
       <c r="L41" t="n">
-        <v>0.61</v>
+        <v>0.58</v>
       </c>
       <c r="M41" t="n">
-        <v>4.85</v>
+        <v>4.6</v>
       </c>
       <c r="N41" t="n">
-        <v>-3.07</v>
+        <v>-2.92</v>
       </c>
       <c r="O41" t="n">
-        <v>4.7</v>
+        <v>4.9</v>
       </c>
       <c r="P41" t="n">
-        <v>7.94</v>
+        <v>7.65</v>
       </c>
       <c r="Q41" t="n">
-        <v>8.98</v>
+        <v>8.66</v>
       </c>
       <c r="R41" t="n">
         <v>5.1</v>
@@ -5992,7 +5992,7 @@
         </is>
       </c>
       <c r="E42" t="n">
-        <v>9593720000</v>
+        <v>9525480000</v>
       </c>
       <c r="F42" t="inlineStr">
         <is>
@@ -6003,34 +6003,34 @@
         <v>2077100000</v>
       </c>
       <c r="H42" t="n">
-        <v>2.45</v>
+        <v>1.55</v>
       </c>
       <c r="I42" t="n">
         <v>53.27</v>
       </c>
       <c r="J42" t="n">
-        <v>8.06</v>
+        <v>7.99</v>
       </c>
       <c r="K42" t="n">
-        <v>5.02</v>
+        <v>4.97</v>
       </c>
       <c r="L42" t="n">
         <v>0.79</v>
       </c>
       <c r="M42" t="n">
-        <v>4.64</v>
+        <v>4.6</v>
       </c>
       <c r="N42" t="n">
-        <v>-3.42</v>
+        <v>-3.39</v>
       </c>
       <c r="O42" t="n">
         <v>0.8</v>
       </c>
       <c r="P42" t="n">
-        <v>8.789999999999999</v>
+        <v>8.73</v>
       </c>
       <c r="Q42" t="n">
-        <v>10.06</v>
+        <v>9.99</v>
       </c>
       <c r="R42" t="n">
         <v>12.8</v>
@@ -6122,7 +6122,7 @@
         </is>
       </c>
       <c r="E43" t="n">
-        <v>33568400000</v>
+        <v>32685500000</v>
       </c>
       <c r="F43" t="inlineStr">
         <is>
@@ -6133,34 +6133,34 @@
         <v>658883000</v>
       </c>
       <c r="H43" t="n">
-        <v>5.42</v>
+        <v>0.41</v>
       </c>
       <c r="I43" t="n">
         <v>34.32</v>
       </c>
       <c r="J43" t="n">
-        <v>5.18</v>
+        <v>4.94</v>
       </c>
       <c r="K43" t="n">
-        <v>1.95</v>
+        <v>1.86</v>
       </c>
       <c r="L43" t="n">
-        <v>0.39</v>
+        <v>0.37</v>
       </c>
       <c r="M43" t="n">
-        <v>3.84</v>
+        <v>3.66</v>
       </c>
       <c r="N43" t="n">
-        <v>-0.9399999999999999</v>
+        <v>-0.9</v>
       </c>
       <c r="O43" t="n">
-        <v>6.6</v>
+        <v>6.9</v>
       </c>
       <c r="P43" t="n">
-        <v>9.27</v>
+        <v>9.029999999999999</v>
       </c>
       <c r="Q43" t="n">
-        <v>9.359999999999999</v>
+        <v>9.119999999999999</v>
       </c>
       <c r="R43" t="n">
         <v>14.8</v>
@@ -6252,7 +6252,7 @@
         </is>
       </c>
       <c r="E44" t="n">
-        <v>148570000000</v>
+        <v>147337000000</v>
       </c>
       <c r="F44" t="inlineStr">
         <is>
@@ -6263,34 +6263,34 @@
         <v>11213700000</v>
       </c>
       <c r="H44" t="n">
-        <v>11.14</v>
+        <v>10.37</v>
       </c>
       <c r="I44" t="n">
         <v>58.33</v>
       </c>
       <c r="J44" t="n">
-        <v>379.79</v>
+        <v>376.54</v>
       </c>
       <c r="K44" t="n">
-        <v>17.25</v>
+        <v>17.11</v>
       </c>
       <c r="L44" t="n">
-        <v>1.26</v>
+        <v>1.25</v>
       </c>
       <c r="M44" t="n">
-        <v>19.57</v>
+        <v>19.4</v>
       </c>
       <c r="N44" t="n">
-        <v>-21.13</v>
+        <v>-20.95</v>
       </c>
       <c r="O44" t="n">
-        <v>9.5</v>
+        <v>9.6</v>
       </c>
       <c r="P44" t="n">
-        <v>88.28</v>
+        <v>87.54000000000001</v>
       </c>
       <c r="Q44" t="n">
-        <v>390.97</v>
+        <v>387.73</v>
       </c>
       <c r="R44" t="n">
         <v>-0.2</v>
@@ -6395,7 +6395,7 @@
         <v>11026900000</v>
       </c>
       <c r="H45" t="n">
-        <v>1.2</v>
+        <v>1.02</v>
       </c>
       <c r="I45" t="n">
         <v>62.4</v>
@@ -6536,7 +6536,7 @@
         </is>
       </c>
       <c r="E46" t="n">
-        <v>45248900000</v>
+        <v>45473600000</v>
       </c>
       <c r="F46" t="inlineStr">
         <is>
@@ -6547,34 +6547,34 @@
         <v>6241480000</v>
       </c>
       <c r="H46" t="n">
-        <v>-12.26</v>
+        <v>-11.3</v>
       </c>
       <c r="I46" t="n">
         <v>-10.61</v>
       </c>
       <c r="J46" t="n">
-        <v>6.65</v>
+        <v>6.72</v>
       </c>
       <c r="K46" t="n">
-        <v>0.99</v>
+        <v>1</v>
       </c>
       <c r="L46" t="n">
         <v>0.33</v>
       </c>
       <c r="M46" t="n">
-        <v>2.92</v>
+        <v>2.95</v>
       </c>
       <c r="N46" t="n">
         <v>-0.68</v>
       </c>
       <c r="O46" t="n">
-        <v>8.6</v>
+        <v>8.5</v>
       </c>
       <c r="P46" t="n">
-        <v>5.7</v>
+        <v>5.72</v>
       </c>
       <c r="Q46" t="n">
-        <v>14.65</v>
+        <v>14.72</v>
       </c>
       <c r="R46" t="n">
         <v>3.4</v>
@@ -6666,7 +6666,7 @@
         </is>
       </c>
       <c r="E47" t="n">
-        <v>13718700000</v>
+        <v>13668300000</v>
       </c>
       <c r="F47" t="inlineStr">
         <is>
@@ -6677,13 +6677,13 @@
         <v>1006840000</v>
       </c>
       <c r="H47" t="n">
-        <v>13.38</v>
+        <v>13</v>
       </c>
       <c r="I47" t="n">
         <v>16.34</v>
       </c>
       <c r="J47" t="n">
-        <v>4.14</v>
+        <v>4.13</v>
       </c>
       <c r="K47" t="n">
         <v>0.95</v>
@@ -6692,19 +6692,19 @@
         <v>0.8</v>
       </c>
       <c r="M47" t="n">
-        <v>3.17</v>
+        <v>3.16</v>
       </c>
       <c r="N47" t="n">
-        <v>6.2</v>
+        <v>6.18</v>
       </c>
       <c r="O47" t="n">
-        <v>5.9</v>
+        <v>6</v>
       </c>
       <c r="P47" t="n">
-        <v>2.76</v>
+        <v>2.75</v>
       </c>
       <c r="Q47" t="n">
-        <v>3.75</v>
+        <v>3.73</v>
       </c>
       <c r="R47" t="n">
         <v>7.6</v>
@@ -6796,7 +6796,7 @@
         </is>
       </c>
       <c r="E48" t="n">
-        <v>72930700000</v>
+        <v>71851200000</v>
       </c>
       <c r="F48" t="inlineStr">
         <is>
@@ -6807,34 +6807,34 @@
         <v>1401920000</v>
       </c>
       <c r="H48" t="n">
-        <v>-16.92</v>
+        <v>-20.77</v>
       </c>
       <c r="I48" t="n">
         <v>31.22</v>
       </c>
       <c r="J48" t="n">
-        <v>4</v>
+        <v>3.82</v>
       </c>
       <c r="K48" t="n">
         <v>0.14</v>
       </c>
       <c r="L48" t="n">
-        <v>0.17</v>
+        <v>0.16</v>
       </c>
       <c r="M48" t="n">
-        <v>6.39</v>
+        <v>6.09</v>
       </c>
       <c r="N48" t="n">
-        <v>-0.32</v>
+        <v>-0.31</v>
       </c>
       <c r="O48" t="n">
-        <v>10.4</v>
+        <v>10.9</v>
       </c>
       <c r="P48" t="n">
-        <v>5.67</v>
+        <v>5.59</v>
       </c>
       <c r="Q48" t="n">
-        <v>12.54</v>
+        <v>12.35</v>
       </c>
       <c r="R48" t="n">
         <v>13.9</v>
@@ -6926,7 +6926,7 @@
         </is>
       </c>
       <c r="E49" t="n">
-        <v>8579830000</v>
+        <v>7951310000</v>
       </c>
       <c r="F49" t="inlineStr">
         <is>
@@ -6937,34 +6937,34 @@
         <v>775945000</v>
       </c>
       <c r="H49" t="n">
-        <v>-25.14</v>
+        <v>-34.29</v>
       </c>
       <c r="I49" t="n">
         <v>48.76</v>
       </c>
       <c r="J49" t="n">
-        <v>3.42</v>
+        <v>3</v>
       </c>
       <c r="K49" t="n">
-        <v>0.13</v>
+        <v>0.12</v>
       </c>
       <c r="L49" t="n">
-        <v>0.14</v>
+        <v>0.12</v>
       </c>
       <c r="M49" t="n">
-        <v>2.43</v>
+        <v>2.13</v>
       </c>
       <c r="N49" t="n">
-        <v>-0.73</v>
+        <v>-0.64</v>
       </c>
       <c r="O49" t="n">
-        <v>1.2</v>
+        <v>1.4</v>
       </c>
       <c r="P49" t="n">
-        <v>3.07</v>
+        <v>2.84</v>
       </c>
       <c r="Q49" t="n">
-        <v>5.7</v>
+        <v>5.29</v>
       </c>
       <c r="R49" t="n">
         <v>1.6</v>
@@ -7056,7 +7056,7 @@
         </is>
       </c>
       <c r="E50" t="n">
-        <v>60107000000</v>
+        <v>59359600000</v>
       </c>
       <c r="F50" t="inlineStr">
         <is>
@@ -7067,34 +7067,34 @@
         <v>2020000000</v>
       </c>
       <c r="H50" t="n">
-        <v>-3.37</v>
+        <v>-5.84</v>
       </c>
       <c r="I50" t="n">
         <v>53.47</v>
       </c>
       <c r="J50" t="n">
-        <v>4.19</v>
+        <v>4.09</v>
       </c>
       <c r="K50" t="n">
-        <v>1.57</v>
+        <v>1.53</v>
       </c>
       <c r="L50" t="n">
-        <v>0.39</v>
+        <v>0.38</v>
       </c>
       <c r="M50" t="n">
-        <v>2.93</v>
+        <v>2.85</v>
       </c>
       <c r="N50" t="n">
-        <v>-0.92</v>
+        <v>-0.9</v>
       </c>
       <c r="O50" t="n">
         <v>2.7</v>
       </c>
       <c r="P50" t="n">
-        <v>7</v>
+        <v>6.92</v>
       </c>
       <c r="Q50" t="n">
-        <v>8.609999999999999</v>
+        <v>8.5</v>
       </c>
       <c r="R50" t="n">
         <v>5.7</v>
@@ -7186,7 +7186,7 @@
         </is>
       </c>
       <c r="E51" t="n">
-        <v>11325200000</v>
+        <v>11150700000</v>
       </c>
       <c r="F51" t="inlineStr">
         <is>
@@ -7197,34 +7197,34 @@
         <v>562836000</v>
       </c>
       <c r="H51" t="n">
-        <v>-22.59</v>
+        <v>-26.57</v>
       </c>
       <c r="I51" t="n">
         <v>46.7</v>
       </c>
       <c r="J51" t="n">
-        <v>1.92</v>
+        <v>1.82</v>
       </c>
       <c r="K51" t="n">
-        <v>0.3</v>
+        <v>0.28</v>
       </c>
       <c r="L51" t="n">
-        <v>0.12</v>
+        <v>0.11</v>
       </c>
       <c r="M51" t="n">
-        <v>0.42</v>
+        <v>0.4</v>
       </c>
       <c r="N51" t="n">
-        <v>-0.49</v>
+        <v>-0.46</v>
       </c>
       <c r="O51" t="n">
         <v>0</v>
       </c>
       <c r="P51" t="n">
-        <v>5.64</v>
+        <v>5.55</v>
       </c>
       <c r="Q51" t="n">
-        <v>6.41</v>
+        <v>6.32</v>
       </c>
       <c r="R51" t="n">
         <v>13.5</v>
@@ -7316,7 +7316,7 @@
         </is>
       </c>
       <c r="E52" t="n">
-        <v>19697400000</v>
+        <v>19543500000</v>
       </c>
       <c r="F52" t="inlineStr">
         <is>
@@ -7327,34 +7327,34 @@
         <v>513164000</v>
       </c>
       <c r="H52" t="n">
-        <v>9.460000000000001</v>
+        <v>8.35</v>
       </c>
       <c r="I52" t="n">
         <v>35.84</v>
       </c>
       <c r="J52" t="n">
-        <v>7.29</v>
+        <v>7.21</v>
       </c>
       <c r="K52" t="n">
-        <v>5</v>
+        <v>4.95</v>
       </c>
       <c r="L52" t="n">
-        <v>1.14</v>
+        <v>1.13</v>
       </c>
       <c r="M52" t="n">
-        <v>43.74</v>
+        <v>43.3</v>
       </c>
       <c r="N52" t="n">
-        <v>-3.21</v>
+        <v>-3.18</v>
       </c>
       <c r="O52" t="n">
         <v>3.7</v>
       </c>
       <c r="P52" t="n">
-        <v>8.880000000000001</v>
+        <v>8.81</v>
       </c>
       <c r="Q52" t="n">
-        <v>9.449999999999999</v>
+        <v>9.380000000000001</v>
       </c>
       <c r="R52" t="n">
         <v>19.9</v>
@@ -7446,7 +7446,7 @@
         </is>
       </c>
       <c r="E53" t="n">
-        <v>17879600000</v>
+        <v>17522200000</v>
       </c>
       <c r="F53" t="inlineStr">
         <is>
@@ -7457,34 +7457,34 @@
         <v>1374560000</v>
       </c>
       <c r="H53" t="n">
-        <v>35.57</v>
+        <v>32.08</v>
       </c>
       <c r="I53" t="n">
         <v>-26.89</v>
       </c>
       <c r="J53" t="n">
-        <v>5.64</v>
+        <v>5.5</v>
       </c>
       <c r="K53" t="n">
-        <v>0.64</v>
+        <v>0.62</v>
       </c>
       <c r="L53" t="n">
-        <v>0.5</v>
+        <v>0.48</v>
       </c>
       <c r="M53" t="n">
-        <v>3.05</v>
+        <v>2.97</v>
       </c>
       <c r="N53" t="n">
-        <v>-3.59</v>
+        <v>-3.5</v>
       </c>
       <c r="O53" t="n">
         <v>0</v>
       </c>
       <c r="P53" t="n">
-        <v>5.38</v>
+        <v>5.27</v>
       </c>
       <c r="Q53" t="n">
-        <v>7.27</v>
+        <v>7.12</v>
       </c>
       <c r="R53" t="n">
         <v>1.8</v>
@@ -7576,7 +7576,7 @@
         </is>
       </c>
       <c r="E54" t="n">
-        <v>970461000000</v>
+        <v>934244000000</v>
       </c>
       <c r="F54" t="inlineStr">
         <is>
@@ -7587,34 +7587,34 @@
         <v>12888700000</v>
       </c>
       <c r="H54" t="n">
-        <v>55.55</v>
+        <v>46.84</v>
       </c>
       <c r="I54" t="n">
         <v>-9.4</v>
       </c>
       <c r="J54" t="n">
+        <v>3.14</v>
+      </c>
+      <c r="K54" t="n">
+        <v>1.22</v>
+      </c>
+      <c r="L54" t="n">
+        <v>0.49</v>
+      </c>
+      <c r="M54" t="n">
+        <v>-12.55</v>
+      </c>
+      <c r="N54" t="n">
+        <v>-0.93</v>
+      </c>
+      <c r="O54" t="n">
+        <v>6.7</v>
+      </c>
+      <c r="P54" t="n">
         <v>3.32</v>
       </c>
-      <c r="K54" t="n">
-        <v>1.3</v>
-      </c>
-      <c r="L54" t="n">
-        <v>0.52</v>
-      </c>
-      <c r="M54" t="n">
-        <v>-13.29</v>
-      </c>
-      <c r="N54" t="n">
-        <v>-0.98</v>
-      </c>
-      <c r="O54" t="n">
-        <v>6.3</v>
-      </c>
-      <c r="P54" t="n">
-        <v>3.45</v>
-      </c>
       <c r="Q54" t="n">
-        <v>4.99</v>
+        <v>4.8</v>
       </c>
       <c r="R54" t="n">
         <v>-2.9</v>
@@ -7706,7 +7706,7 @@
         </is>
       </c>
       <c r="E55" t="n">
-        <v>897382000000</v>
+        <v>870187000000</v>
       </c>
       <c r="F55" t="inlineStr">
         <is>
@@ -7717,34 +7717,34 @@
         <v>12888700000</v>
       </c>
       <c r="H55" t="n">
-        <v>45.96</v>
+        <v>39.04</v>
       </c>
       <c r="I55" t="n">
         <v>-6.06</v>
       </c>
       <c r="J55" t="n">
-        <v>2.95</v>
+        <v>2.81</v>
       </c>
       <c r="K55" t="n">
-        <v>1.15</v>
+        <v>1.1</v>
       </c>
       <c r="L55" t="n">
-        <v>0.46</v>
+        <v>0.44</v>
       </c>
       <c r="M55" t="n">
-        <v>-11.79</v>
+        <v>-11.23</v>
       </c>
       <c r="N55" t="n">
-        <v>-0.87</v>
+        <v>-0.83</v>
       </c>
       <c r="O55" t="n">
-        <v>7.1</v>
+        <v>7.5</v>
       </c>
       <c r="P55" t="n">
-        <v>3.19</v>
+        <v>3.09</v>
       </c>
       <c r="Q55" t="n">
-        <v>4.61</v>
+        <v>4.47</v>
       </c>
       <c r="R55" t="n">
         <v>-2.9</v>
@@ -7836,7 +7836,7 @@
         </is>
       </c>
       <c r="E56" t="n">
-        <v>8959790000</v>
+        <v>9197270000</v>
       </c>
       <c r="F56" t="inlineStr">
         <is>
@@ -7847,34 +7847,34 @@
         <v>1249900000</v>
       </c>
       <c r="H56" t="n">
-        <v>0.38</v>
+        <v>3.6</v>
       </c>
       <c r="I56" t="n">
         <v>5.31</v>
       </c>
       <c r="J56" t="n">
-        <v>5.2</v>
+        <v>5.37</v>
       </c>
       <c r="K56" t="n">
-        <v>0.82</v>
+        <v>0.85</v>
       </c>
       <c r="L56" t="n">
-        <v>0.78</v>
+        <v>0.8</v>
       </c>
       <c r="M56" t="n">
-        <v>2.68</v>
+        <v>2.76</v>
       </c>
       <c r="N56" t="n">
-        <v>29.82</v>
+        <v>30.78</v>
       </c>
       <c r="O56" t="n">
-        <v>15.9</v>
+        <v>15.4</v>
       </c>
       <c r="P56" t="n">
-        <v>5.65</v>
+        <v>5.8</v>
       </c>
       <c r="Q56" t="n">
-        <v>6.29</v>
+        <v>6.46</v>
       </c>
       <c r="R56" t="n">
         <v>24.2</v>
@@ -7966,7 +7966,7 @@
         </is>
       </c>
       <c r="E57" t="n">
-        <v>83786600000</v>
+        <v>78918100000</v>
       </c>
       <c r="F57" t="inlineStr">
         <is>
@@ -7977,34 +7977,34 @@
         <v>872495000</v>
       </c>
       <c r="H57" t="n">
-        <v>65.14</v>
+        <v>51.67</v>
       </c>
       <c r="I57" t="n">
         <v>3.16</v>
       </c>
       <c r="J57" t="n">
-        <v>15.86</v>
+        <v>14.56</v>
       </c>
       <c r="K57" t="n">
-        <v>3.38</v>
+        <v>3.1</v>
       </c>
       <c r="L57" t="n">
-        <v>0.9399999999999999</v>
+        <v>0.86</v>
       </c>
       <c r="M57" t="n">
-        <v>11.69</v>
+        <v>10.74</v>
       </c>
       <c r="N57" t="n">
-        <v>-2.27</v>
+        <v>-2.09</v>
       </c>
       <c r="O57" t="n">
         <v>0</v>
       </c>
       <c r="P57" t="n">
-        <v>8.369999999999999</v>
+        <v>7.89</v>
       </c>
       <c r="Q57" t="n">
-        <v>22.26</v>
+        <v>20.97</v>
       </c>
       <c r="R57" t="n">
         <v>36.8</v>
@@ -8096,7 +8096,7 @@
         </is>
       </c>
       <c r="E58" t="n">
-        <v>18751500000</v>
+        <v>17995000000</v>
       </c>
       <c r="F58" t="inlineStr">
         <is>
@@ -8107,34 +8107,34 @@
         <v>646586000</v>
       </c>
       <c r="H58" t="n">
-        <v>4.42</v>
+        <v>1.94</v>
       </c>
       <c r="I58" t="n">
         <v>40.5</v>
       </c>
       <c r="J58" t="n">
-        <v>0.92</v>
+        <v>0.9</v>
       </c>
       <c r="K58" t="n">
-        <v>0.76</v>
+        <v>0.74</v>
       </c>
       <c r="L58" t="n">
-        <v>0.55</v>
+        <v>0.54</v>
       </c>
       <c r="M58" t="n">
-        <v>4.79</v>
+        <v>4.68</v>
       </c>
       <c r="N58" t="n">
-        <v>-4.12</v>
+        <v>-4.02</v>
       </c>
       <c r="O58" t="n">
-        <v>6.1</v>
+        <v>6.2</v>
       </c>
       <c r="P58" t="n">
-        <v>0.54</v>
+        <v>0.52</v>
       </c>
       <c r="Q58" t="n">
-        <v>0.54</v>
+        <v>0.52</v>
       </c>
       <c r="R58" t="n">
         <v>15.8</v>
@@ -8226,7 +8226,7 @@
         </is>
       </c>
       <c r="E59" t="n">
-        <v>34999400000</v>
+        <v>34421100000</v>
       </c>
       <c r="F59" t="inlineStr">
         <is>
@@ -8237,34 +8237,34 @@
         <v>1752370000</v>
       </c>
       <c r="H59" t="n">
-        <v>-22.18</v>
+        <v>-23.59</v>
       </c>
       <c r="I59" t="n">
         <v>10.98</v>
       </c>
       <c r="J59" t="n">
-        <v>11.19</v>
+        <v>10.98</v>
       </c>
       <c r="K59" t="n">
-        <v>0.71</v>
+        <v>0.7</v>
       </c>
       <c r="L59" t="n">
-        <v>1.26</v>
+        <v>1.24</v>
       </c>
       <c r="M59" t="n">
-        <v>6.5</v>
+        <v>6.39</v>
       </c>
       <c r="N59" t="n">
-        <v>-12.38</v>
+        <v>-12.15</v>
       </c>
       <c r="O59" t="n">
         <v>2.2</v>
       </c>
       <c r="P59" t="n">
-        <v>7.14</v>
+        <v>7.02</v>
       </c>
       <c r="Q59" t="n">
-        <v>12.28</v>
+        <v>12.08</v>
       </c>
       <c r="R59" t="n">
         <v>15.4</v>
@@ -8356,7 +8356,7 @@
         </is>
       </c>
       <c r="E60" t="n">
-        <v>43880400000</v>
+        <v>43341400000</v>
       </c>
       <c r="F60" t="inlineStr">
         <is>
@@ -8367,34 +8367,34 @@
         <v>1858830000</v>
       </c>
       <c r="H60" t="n">
-        <v>-3.05</v>
+        <v>-5.03</v>
       </c>
       <c r="I60" t="n">
         <v>-13.67</v>
       </c>
       <c r="J60" t="n">
-        <v>4.6</v>
+        <v>4.51</v>
       </c>
       <c r="K60" t="n">
-        <v>1.86</v>
+        <v>1.83</v>
       </c>
       <c r="L60" t="n">
-        <v>0.49</v>
+        <v>0.48</v>
       </c>
       <c r="M60" t="n">
-        <v>11.66</v>
+        <v>11.42</v>
       </c>
       <c r="N60" t="n">
-        <v>-0.84</v>
+        <v>-0.83</v>
       </c>
       <c r="O60" t="n">
-        <v>6.5</v>
+        <v>6.6</v>
       </c>
       <c r="P60" t="n">
-        <v>5.75</v>
+        <v>5.68</v>
       </c>
       <c r="Q60" t="n">
-        <v>7.64</v>
+        <v>7.55</v>
       </c>
       <c r="R60" t="n">
         <v>16</v>
@@ -8486,7 +8486,7 @@
         </is>
       </c>
       <c r="E61" t="n">
-        <v>85250300000</v>
+        <v>84792400000</v>
       </c>
       <c r="F61" t="inlineStr">
         <is>
@@ -8497,34 +8497,34 @@
         <v>2289290000</v>
       </c>
       <c r="H61" t="n">
-        <v>-15.81</v>
+        <v>-16.3</v>
       </c>
       <c r="I61" t="n">
         <v>76.31999999999999</v>
       </c>
       <c r="J61" t="n">
-        <v>7.66</v>
+        <v>7.62</v>
       </c>
       <c r="K61" t="n">
-        <v>1.37</v>
+        <v>1.36</v>
       </c>
       <c r="L61" t="n">
         <v>0.71</v>
       </c>
       <c r="M61" t="n">
-        <v>2.19</v>
+        <v>2.17</v>
       </c>
       <c r="N61" t="n">
-        <v>-2.39</v>
+        <v>-2.37</v>
       </c>
       <c r="O61" t="n">
-        <v>12.5</v>
+        <v>12.6</v>
       </c>
       <c r="P61" t="n">
-        <v>7.08</v>
+        <v>7.04</v>
       </c>
       <c r="Q61" t="n">
-        <v>8.380000000000001</v>
+        <v>8.33</v>
       </c>
       <c r="R61" t="n">
         <v>29.3</v>
@@ -8616,7 +8616,7 @@
         </is>
       </c>
       <c r="E62" t="n">
-        <v>5129200000</v>
+        <v>4809430000</v>
       </c>
       <c r="F62" t="inlineStr">
         <is>
@@ -8624,37 +8624,37 @@
         </is>
       </c>
       <c r="G62" t="n">
-        <v>293472000</v>
+        <v>293482000</v>
       </c>
       <c r="H62" t="n">
-        <v>22.66</v>
+        <v>11.8</v>
       </c>
       <c r="I62" t="n">
         <v>-26.43</v>
       </c>
       <c r="J62" t="n">
-        <v>5.37</v>
+        <v>4.89</v>
       </c>
       <c r="K62" t="n">
-        <v>1.21</v>
+        <v>1.1</v>
       </c>
       <c r="L62" t="n">
-        <v>0.4</v>
+        <v>0.36</v>
       </c>
       <c r="M62" t="n">
-        <v>2.97</v>
+        <v>2.71</v>
       </c>
       <c r="N62" t="n">
-        <v>-1.38</v>
+        <v>-1.25</v>
       </c>
       <c r="O62" t="n">
-        <v>11.1</v>
+        <v>12.2</v>
       </c>
       <c r="P62" t="n">
-        <v>3.69</v>
+        <v>3.46</v>
       </c>
       <c r="Q62" t="n">
-        <v>7.62</v>
+        <v>7.15</v>
       </c>
       <c r="R62" t="n">
         <v>16.2</v>
@@ -8746,7 +8746,7 @@
         </is>
       </c>
       <c r="E63" t="n">
-        <v>81029600000</v>
+        <v>78769900000</v>
       </c>
       <c r="F63" t="inlineStr">
         <is>
@@ -8757,34 +8757,34 @@
         <v>1124260000</v>
       </c>
       <c r="H63" t="n">
-        <v>0.45</v>
+        <v>-4.21</v>
       </c>
       <c r="I63" t="n">
         <v>46.65</v>
       </c>
       <c r="J63" t="n">
-        <v>5.94</v>
+        <v>5.67</v>
       </c>
       <c r="K63" t="n">
-        <v>1.11</v>
+        <v>1.06</v>
       </c>
       <c r="L63" t="n">
-        <v>0.57</v>
+        <v>0.54</v>
       </c>
       <c r="M63" t="n">
-        <v>12.99</v>
+        <v>12.39</v>
       </c>
       <c r="N63" t="n">
-        <v>-1.25</v>
+        <v>-1.19</v>
       </c>
       <c r="O63" t="n">
-        <v>4.6</v>
+        <v>4.8</v>
       </c>
       <c r="P63" t="n">
-        <v>5.68</v>
+        <v>5.52</v>
       </c>
       <c r="Q63" t="n">
-        <v>9.880000000000001</v>
+        <v>9.609999999999999</v>
       </c>
       <c r="R63" t="n">
         <v>40.1</v>
@@ -8889,7 +8889,7 @@
         <v>7498530000</v>
       </c>
       <c r="H64" t="n">
-        <v>-17.91</v>
+        <v>-17.58</v>
       </c>
       <c r="I64" t="n">
         <v>51.61</v>
@@ -9030,7 +9030,7 @@
         </is>
       </c>
       <c r="E65" t="n">
-        <v>132769000000</v>
+        <v>128610000000</v>
       </c>
       <c r="F65" t="inlineStr">
         <is>
@@ -9041,34 +9041,34 @@
         <v>3524530000</v>
       </c>
       <c r="H65" t="n">
-        <v>7.34</v>
+        <v>2.89</v>
       </c>
       <c r="I65" t="n">
         <v>62.39</v>
       </c>
       <c r="J65" t="n">
-        <v>7.8</v>
+        <v>7.48</v>
       </c>
       <c r="K65" t="n">
-        <v>2.53</v>
+        <v>2.43</v>
       </c>
       <c r="L65" t="n">
-        <v>0.86</v>
+        <v>0.82</v>
       </c>
       <c r="M65" t="n">
-        <v>9.1</v>
+        <v>8.720000000000001</v>
       </c>
       <c r="N65" t="n">
-        <v>-2.14</v>
+        <v>-2.05</v>
       </c>
       <c r="O65" t="n">
-        <v>2.4</v>
+        <v>2.5</v>
       </c>
       <c r="P65" t="n">
-        <v>8.75</v>
+        <v>8.470000000000001</v>
       </c>
       <c r="Q65" t="n">
-        <v>10.33</v>
+        <v>10</v>
       </c>
       <c r="R65" t="n">
         <v>21</v>
@@ -9160,7 +9160,7 @@
         </is>
       </c>
       <c r="E66" t="n">
-        <v>14361600000</v>
+        <v>13932700000</v>
       </c>
       <c r="F66" t="inlineStr">
         <is>
@@ -9171,34 +9171,34 @@
         <v>498746000</v>
       </c>
       <c r="H66" t="n">
-        <v>12.63</v>
+        <v>6.6</v>
       </c>
       <c r="I66" t="n">
         <v>-0.5600000000000001</v>
       </c>
       <c r="J66" t="n">
-        <v>4.6</v>
+        <v>4.35</v>
       </c>
       <c r="K66" t="n">
-        <v>0.84</v>
+        <v>0.79</v>
       </c>
       <c r="L66" t="n">
-        <v>0.4</v>
+        <v>0.38</v>
       </c>
       <c r="M66" t="n">
-        <v>1.73</v>
+        <v>1.64</v>
       </c>
       <c r="N66" t="n">
-        <v>-1.5</v>
+        <v>-1.42</v>
       </c>
       <c r="O66" t="n">
-        <v>5</v>
+        <v>5.3</v>
       </c>
       <c r="P66" t="n">
-        <v>6.8</v>
+        <v>6.59</v>
       </c>
       <c r="Q66" t="n">
-        <v>8.23</v>
+        <v>7.99</v>
       </c>
       <c r="R66" t="n">
         <v>2.4</v>
@@ -9290,7 +9290,7 @@
         </is>
       </c>
       <c r="E67" t="n">
-        <v>15778700000</v>
+        <v>15409000000</v>
       </c>
       <c r="F67" t="inlineStr">
         <is>
@@ -9301,34 +9301,34 @@
         <v>616130000</v>
       </c>
       <c r="H67" t="n">
-        <v>-18.44</v>
+        <v>-21.02</v>
       </c>
       <c r="I67" t="n">
         <v>43.23</v>
       </c>
       <c r="J67" t="n">
-        <v>6.38</v>
+        <v>6.18</v>
       </c>
       <c r="K67" t="n">
-        <v>1.52</v>
+        <v>1.47</v>
       </c>
       <c r="L67" t="n">
-        <v>0.52</v>
+        <v>0.5</v>
       </c>
       <c r="M67" t="n">
-        <v>4.61</v>
+        <v>4.46</v>
       </c>
       <c r="N67" t="n">
-        <v>-1.09</v>
+        <v>-1.06</v>
       </c>
       <c r="O67" t="n">
-        <v>5.3</v>
+        <v>5.5</v>
       </c>
       <c r="P67" t="n">
-        <v>4.29</v>
+        <v>4.19</v>
       </c>
       <c r="Q67" t="n">
-        <v>8.630000000000001</v>
+        <v>8.43</v>
       </c>
       <c r="R67" t="n">
         <v>51.5</v>
@@ -9420,7 +9420,7 @@
         </is>
       </c>
       <c r="E68" t="n">
-        <v>121100000000</v>
+        <v>119772000000</v>
       </c>
       <c r="F68" t="inlineStr">
         <is>
@@ -9431,34 +9431,34 @@
         <v>1264120000</v>
       </c>
       <c r="H68" t="n">
-        <v>-18.95</v>
+        <v>-20.99</v>
       </c>
       <c r="I68" t="n">
         <v>-14.91</v>
       </c>
       <c r="J68" t="n">
-        <v>5.58</v>
+        <v>5.44</v>
       </c>
       <c r="K68" t="n">
-        <v>1.06</v>
+        <v>1.04</v>
       </c>
       <c r="L68" t="n">
-        <v>0.32</v>
+        <v>0.31</v>
       </c>
       <c r="M68" t="n">
-        <v>1.74</v>
+        <v>1.7</v>
       </c>
       <c r="N68" t="n">
-        <v>-0.7</v>
+        <v>-0.68</v>
       </c>
       <c r="O68" t="n">
         <v>0</v>
       </c>
       <c r="P68" t="n">
-        <v>5.75</v>
+        <v>5.69</v>
       </c>
       <c r="Q68" t="n">
-        <v>12.81</v>
+        <v>12.67</v>
       </c>
       <c r="R68" t="n">
         <v>3.1</v>
@@ -9550,7 +9550,7 @@
         </is>
       </c>
       <c r="E69" t="n">
-        <v>23421700000</v>
+        <v>23480300000</v>
       </c>
       <c r="F69" t="inlineStr">
         <is>
@@ -9561,34 +9561,34 @@
         <v>1033500000</v>
       </c>
       <c r="H69" t="n">
-        <v>-4.96</v>
+        <v>-4.54</v>
       </c>
       <c r="I69" t="n">
         <v>38.85</v>
       </c>
       <c r="J69" t="n">
-        <v>5.83</v>
+        <v>5.86</v>
       </c>
       <c r="K69" t="n">
-        <v>2.85</v>
+        <v>2.86</v>
       </c>
       <c r="L69" t="n">
-        <v>0.57</v>
+        <v>0.58</v>
       </c>
       <c r="M69" t="n">
-        <v>6.13</v>
+        <v>6.15</v>
       </c>
       <c r="N69" t="n">
         <v>-1.17</v>
       </c>
       <c r="O69" t="n">
-        <v>8.5</v>
+        <v>8.4</v>
       </c>
       <c r="P69" t="n">
-        <v>9.9</v>
+        <v>9.92</v>
       </c>
       <c r="Q69" t="n">
-        <v>10.24</v>
+        <v>10.26</v>
       </c>
       <c r="R69" t="n">
         <v>11.8</v>
@@ -9680,7 +9680,7 @@
         </is>
       </c>
       <c r="E70" t="n">
-        <v>50783500000</v>
+        <v>49061200000</v>
       </c>
       <c r="F70" t="inlineStr">
         <is>
@@ -9691,34 +9691,34 @@
         <v>2392130000</v>
       </c>
       <c r="H70" t="n">
-        <v>5.96</v>
+        <v>2.57</v>
       </c>
       <c r="I70" t="n">
         <v>66.08</v>
       </c>
       <c r="J70" t="n">
-        <v>281.95</v>
+        <v>272.92</v>
       </c>
       <c r="K70" t="n">
-        <v>130.48</v>
+        <v>126.3</v>
       </c>
       <c r="L70" t="n">
-        <v>0.93</v>
+        <v>0.9</v>
       </c>
       <c r="M70" t="n">
-        <v>-41.56</v>
+        <v>-40.23</v>
       </c>
       <c r="N70" t="n">
-        <v>-2.79</v>
+        <v>-2.7</v>
       </c>
       <c r="O70" t="n">
-        <v>6.4</v>
+        <v>6.6</v>
       </c>
       <c r="P70" t="n">
-        <v>276.56</v>
+        <v>267.18</v>
       </c>
       <c r="Q70" t="n">
-        <v>266.03</v>
+        <v>257</v>
       </c>
       <c r="R70" t="n">
         <v>-69.59999999999999</v>
@@ -9810,7 +9810,7 @@
         </is>
       </c>
       <c r="E71" t="n">
-        <v>22305200000</v>
+        <v>24109400000</v>
       </c>
       <c r="F71" t="inlineStr">
         <is>
@@ -9821,34 +9821,34 @@
         <v>599402000</v>
       </c>
       <c r="H71" t="n">
-        <v>-24.85</v>
+        <v>-17.66</v>
       </c>
       <c r="I71" t="n">
         <v>59.29</v>
       </c>
       <c r="J71" t="n">
-        <v>8.24</v>
+        <v>9.029999999999999</v>
       </c>
       <c r="K71" t="n">
-        <v>3.14</v>
+        <v>3.44</v>
       </c>
       <c r="L71" t="n">
-        <v>1.45</v>
+        <v>1.58</v>
       </c>
       <c r="M71" t="n">
-        <v>13.02</v>
+        <v>14.27</v>
       </c>
       <c r="N71" t="n">
-        <v>-4.77</v>
+        <v>-5.23</v>
       </c>
       <c r="O71" t="n">
-        <v>2.1</v>
+        <v>1.9</v>
       </c>
       <c r="P71" t="n">
-        <v>8.42</v>
+        <v>9.1</v>
       </c>
       <c r="Q71" t="n">
-        <v>9.74</v>
+        <v>10.53</v>
       </c>
       <c r="R71" t="n">
         <v>15.1</v>
@@ -9940,7 +9940,7 @@
         </is>
       </c>
       <c r="E72" t="n">
-        <v>45988400000</v>
+        <v>42317300000</v>
       </c>
       <c r="F72" t="inlineStr">
         <is>
@@ -9951,34 +9951,34 @@
         <v>1115850000</v>
       </c>
       <c r="H72" t="n">
-        <v>37.32</v>
+        <v>21.58</v>
       </c>
       <c r="I72" t="n">
         <v>44.34</v>
       </c>
       <c r="J72" t="n">
-        <v>5.9</v>
+        <v>5.23</v>
       </c>
       <c r="K72" t="n">
-        <v>0.22</v>
+        <v>0.19</v>
       </c>
       <c r="L72" t="n">
-        <v>0.64</v>
+        <v>0.5600000000000001</v>
       </c>
       <c r="M72" t="n">
-        <v>3.85</v>
+        <v>3.41</v>
       </c>
       <c r="N72" t="n">
-        <v>-2.93</v>
+        <v>-2.6</v>
       </c>
       <c r="O72" t="n">
-        <v>4.5</v>
+        <v>5.1</v>
       </c>
       <c r="P72" t="n">
-        <v>6.44</v>
+        <v>5.92</v>
       </c>
       <c r="Q72" t="n">
-        <v>8.48</v>
+        <v>7.8</v>
       </c>
       <c r="R72" t="n">
         <v>4</v>
@@ -10070,7 +10070,7 @@
         </is>
       </c>
       <c r="E73" t="n">
-        <v>12475000000</v>
+        <v>13402200000</v>
       </c>
       <c r="F73" t="inlineStr">
         <is>
@@ -10081,34 +10081,34 @@
         <v>1253080000</v>
       </c>
       <c r="H73" t="n">
-        <v>73.95</v>
+        <v>86.39</v>
       </c>
       <c r="I73" t="n">
         <v>11.84</v>
       </c>
       <c r="J73" t="n">
-        <v>15.28</v>
+        <v>16.37</v>
       </c>
       <c r="K73" t="n">
-        <v>0.51</v>
+        <v>0.55</v>
       </c>
       <c r="L73" t="n">
-        <v>0.37</v>
+        <v>0.4</v>
       </c>
       <c r="M73" t="n">
-        <v>1.02</v>
+        <v>1.09</v>
       </c>
       <c r="N73" t="n">
-        <v>2.63</v>
+        <v>2.82</v>
       </c>
       <c r="O73" t="n">
         <v>0</v>
       </c>
       <c r="P73" t="n">
-        <v>5.96</v>
+        <v>6.4</v>
       </c>
       <c r="Q73" t="n">
-        <v>14.7</v>
+        <v>15.79</v>
       </c>
       <c r="R73" t="n">
         <v>-7.8</v>
@@ -10200,7 +10200,7 @@
         </is>
       </c>
       <c r="E74" t="n">
-        <v>439662000000</v>
+        <v>433447000000</v>
       </c>
       <c r="F74" t="inlineStr">
         <is>
@@ -10211,34 +10211,34 @@
         <v>4439160000</v>
       </c>
       <c r="H74" t="n">
-        <v>15.48</v>
+        <v>13.54</v>
       </c>
       <c r="I74" t="n">
         <v>48.04</v>
       </c>
       <c r="J74" t="n">
-        <v>5.13</v>
+        <v>5.05</v>
       </c>
       <c r="K74" t="n">
-        <v>1.72</v>
+        <v>1.69</v>
       </c>
       <c r="L74" t="n">
-        <v>0.8100000000000001</v>
+        <v>0.79</v>
       </c>
       <c r="M74" t="n">
-        <v>21.81</v>
+        <v>21.44</v>
       </c>
       <c r="N74" t="n">
-        <v>-2.12</v>
+        <v>-2.09</v>
       </c>
       <c r="O74" t="n">
-        <v>6.7</v>
+        <v>6.9</v>
       </c>
       <c r="P74" t="n">
-        <v>4.91</v>
+        <v>4.84</v>
       </c>
       <c r="Q74" t="n">
-        <v>6.12</v>
+        <v>6.03</v>
       </c>
       <c r="R74" t="n">
         <v>-5.3</v>
@@ -10330,7 +10330,7 @@
         </is>
       </c>
       <c r="E75" t="n">
-        <v>15817000000</v>
+        <v>15511500000</v>
       </c>
       <c r="F75" t="inlineStr">
         <is>
@@ -10341,34 +10341,34 @@
         <v>1221830000</v>
       </c>
       <c r="H75" t="n">
-        <v>1.04</v>
+        <v>-6.73</v>
       </c>
       <c r="I75" t="n">
         <v>-29.45</v>
       </c>
       <c r="J75" t="n">
-        <v>1.48</v>
+        <v>1.36</v>
       </c>
       <c r="K75" t="n">
-        <v>0.66</v>
+        <v>0.61</v>
       </c>
       <c r="L75" t="n">
-        <v>0.17</v>
+        <v>0.16</v>
       </c>
       <c r="M75" t="n">
-        <v>1.39</v>
+        <v>1.28</v>
       </c>
       <c r="N75" t="n">
-        <v>-0.29</v>
+        <v>-0.27</v>
       </c>
       <c r="O75" t="n">
-        <v>3.8</v>
+        <v>4.1</v>
       </c>
       <c r="P75" t="n">
-        <v>4.19</v>
+        <v>4.11</v>
       </c>
       <c r="Q75" t="n">
-        <v>5.88</v>
+        <v>5.77</v>
       </c>
       <c r="R75" t="n">
         <v>10.2</v>
@@ -10460,7 +10460,7 @@
         </is>
       </c>
       <c r="E76" t="n">
-        <v>57405000000</v>
+        <v>54001000000</v>
       </c>
       <c r="F76" t="inlineStr">
         <is>
@@ -10471,34 +10471,34 @@
         <v>1198560000</v>
       </c>
       <c r="H76" t="n">
-        <v>30.42</v>
+        <v>19.11</v>
       </c>
       <c r="I76" t="n">
         <v>62.71</v>
       </c>
       <c r="J76" t="n">
-        <v>7.46</v>
+        <v>6.81</v>
       </c>
       <c r="K76" t="n">
-        <v>0.2</v>
+        <v>0.19</v>
       </c>
       <c r="L76" t="n">
-        <v>0.61</v>
+        <v>0.5600000000000001</v>
       </c>
       <c r="M76" t="n">
+        <v>3.19</v>
+      </c>
+      <c r="N76" t="n">
+        <v>-2.17</v>
+      </c>
+      <c r="O76" t="n">
         <v>3.5</v>
       </c>
-      <c r="N76" t="n">
-        <v>-2.37</v>
-      </c>
-      <c r="O76" t="n">
-        <v>3.2</v>
-      </c>
       <c r="P76" t="n">
-        <v>9</v>
+        <v>8.470000000000001</v>
       </c>
       <c r="Q76" t="n">
-        <v>10.91</v>
+        <v>10.26</v>
       </c>
       <c r="R76" t="n">
         <v>5.9</v>
@@ -10590,7 +10590,7 @@
         </is>
       </c>
       <c r="E77" t="n">
-        <v>5445930000</v>
+        <v>5294760000</v>
       </c>
       <c r="F77" t="inlineStr">
         <is>
@@ -10601,34 +10601,34 @@
         <v>236198000</v>
       </c>
       <c r="H77" t="n">
-        <v>-33.24</v>
+        <v>-35.17</v>
       </c>
       <c r="I77" t="n">
         <v>82.31999999999999</v>
       </c>
       <c r="J77" t="n">
-        <v>7.07</v>
+        <v>6.87</v>
       </c>
       <c r="K77" t="n">
-        <v>1.7</v>
+        <v>1.65</v>
       </c>
       <c r="L77" t="n">
-        <v>1.12</v>
+        <v>1.09</v>
       </c>
       <c r="M77" t="n">
-        <v>2.33</v>
+        <v>2.26</v>
       </c>
       <c r="N77" t="n">
-        <v>3.98</v>
+        <v>3.86</v>
       </c>
       <c r="O77" t="n">
-        <v>3.1</v>
+        <v>3.2</v>
       </c>
       <c r="P77" t="n">
-        <v>6.09</v>
+        <v>5.92</v>
       </c>
       <c r="Q77" t="n">
-        <v>7.35</v>
+        <v>7.14</v>
       </c>
       <c r="R77" t="n">
         <v>18.2</v>
@@ -10720,7 +10720,7 @@
         </is>
       </c>
       <c r="E78" t="n">
-        <v>123035000000</v>
+        <v>118001000000</v>
       </c>
       <c r="F78" t="inlineStr">
         <is>
@@ -10731,34 +10731,34 @@
         <v>3226550000</v>
       </c>
       <c r="H78" t="n">
-        <v>5.76</v>
+        <v>5.29</v>
       </c>
       <c r="I78" t="n">
         <v>49.38</v>
       </c>
       <c r="J78" t="n">
-        <v>11.47</v>
+        <v>10.96</v>
       </c>
       <c r="K78" t="n">
-        <v>1.85</v>
+        <v>1.77</v>
       </c>
       <c r="L78" t="n">
-        <v>0.86</v>
+        <v>0.82</v>
       </c>
       <c r="M78" t="n">
-        <v>43.57</v>
+        <v>41.62</v>
       </c>
       <c r="N78" t="n">
-        <v>-3.5</v>
+        <v>-3.34</v>
       </c>
       <c r="O78" t="n">
-        <v>2.8</v>
+        <v>7.3</v>
       </c>
       <c r="P78" t="n">
-        <v>4.94</v>
+        <v>4.74</v>
       </c>
       <c r="Q78" t="n">
-        <v>12.57</v>
+        <v>12.05</v>
       </c>
       <c r="R78" t="n">
         <v>7.8</v>
@@ -10850,7 +10850,7 @@
         </is>
       </c>
       <c r="E79" t="n">
-        <v>176058000000</v>
+        <v>177191000000</v>
       </c>
       <c r="F79" t="inlineStr">
         <is>
@@ -10861,34 +10861,34 @@
         <v>4197320000</v>
       </c>
       <c r="H79" t="n">
-        <v>-11.76</v>
+        <v>-11.2</v>
       </c>
       <c r="I79" t="n">
         <v>-3.19</v>
       </c>
       <c r="J79" t="n">
-        <v>21.07</v>
+        <v>21.2</v>
       </c>
       <c r="K79" t="n">
-        <v>4.46</v>
+        <v>4.49</v>
       </c>
       <c r="L79" t="n">
-        <v>4.13</v>
+        <v>4.16</v>
       </c>
       <c r="M79" t="n">
-        <v>18.53</v>
+        <v>18.65</v>
       </c>
       <c r="N79" t="n">
-        <v>58.86</v>
+        <v>59.23</v>
       </c>
       <c r="O79" t="n">
-        <v>5.1</v>
+        <v>5</v>
       </c>
       <c r="P79" t="n">
-        <v>18.46</v>
+        <v>18.58</v>
       </c>
       <c r="Q79" t="n">
-        <v>20.68</v>
+        <v>20.82</v>
       </c>
       <c r="R79" t="n">
         <v>12.6</v>
@@ -10980,7 +10980,7 @@
         </is>
       </c>
       <c r="E80" t="n">
-        <v>6911350000</v>
+        <v>6881200000</v>
       </c>
       <c r="F80" t="inlineStr">
         <is>
@@ -10991,13 +10991,13 @@
         <v>274089000</v>
       </c>
       <c r="H80" t="n">
-        <v>-21.36</v>
+        <v>-22.27</v>
       </c>
       <c r="I80" t="n">
         <v>55.13</v>
       </c>
       <c r="J80" t="n">
-        <v>2.86</v>
+        <v>2.83</v>
       </c>
       <c r="K80" t="n">
         <v>0.47</v>
@@ -11006,19 +11006,19 @@
         <v>0.27</v>
       </c>
       <c r="M80" t="n">
-        <v>3.5</v>
+        <v>3.46</v>
       </c>
       <c r="N80" t="n">
-        <v>-0.61</v>
+        <v>-0.6</v>
       </c>
       <c r="O80" t="n">
-        <v>5.9</v>
+        <v>6</v>
       </c>
       <c r="P80" t="n">
-        <v>4.01</v>
+        <v>4</v>
       </c>
       <c r="Q80" t="n">
-        <v>7.54</v>
+        <v>7.5</v>
       </c>
       <c r="R80" t="n">
         <v>5.7</v>

</xml_diff>